<commit_message>
Removed payment sections on Invoice Data tab
</commit_message>
<xml_diff>
--- a/gui/template/Teacher Base Template.xlsx
+++ b/gui/template/Teacher Base Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\PycharmProjects\RueLee\Boston Education\bosvoiceton-gui\gui\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\PycharmProjects\RueLee\bosvoiceton-gui\gui\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BDC157D-B917-4830-B24A-9DAA3BB1D03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017B89D4-C528-4ACB-BE9C-6436C6830620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="root" sheetId="3" r:id="rId1"/>
@@ -994,18 +994,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:J32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.5546875" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" customWidth="1"/>
-    <col min="7" max="7" width="22.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="33" thickBot="1">
+    <row r="1" spans="2:10" ht="32.4" thickBot="1">
       <c r="C1" s="7" t="s">
         <v>11</v>
       </c>
@@ -1013,13 +1013,13 @@
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="2:10" ht="19.5" thickBot="1">
+    <row r="2" spans="2:10" ht="18.600000000000001" thickBot="1">
       <c r="F2" s="14" t="s">
         <v>3</v>
       </c>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="2:10" ht="19.5" thickBot="1">
+    <row r="3" spans="2:10" ht="18.600000000000001" thickBot="1">
       <c r="B3" s="29" t="s">
         <v>19</v>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G3" s="22"/>
     </row>
-    <row r="4" spans="2:10" ht="19.5" thickBot="1">
+    <row r="4" spans="2:10" ht="18.600000000000001" thickBot="1">
       <c r="B4" s="29" t="s">
         <v>0</v>
       </c>
@@ -1050,8 +1050,8 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="2:10" ht="15.75" thickBot="1"/>
-    <row r="7" spans="2:10" ht="16.5" thickBot="1">
+    <row r="6" spans="2:10" ht="15" thickBot="1"/>
+    <row r="7" spans="2:10" ht="16.2" thickBot="1">
       <c r="B7" s="44" t="s">
         <v>4</v>
       </c>
@@ -1061,7 +1061,7 @@
       <c r="F7" s="45"/>
       <c r="G7" s="46"/>
     </row>
-    <row r="8" spans="2:10" ht="15.75" thickBot="1">
+    <row r="8" spans="2:10" ht="15" thickBot="1">
       <c r="B8" s="47"/>
       <c r="C8" s="48"/>
       <c r="D8" s="48"/>
@@ -1069,8 +1069,8 @@
       <c r="F8" s="48"/>
       <c r="G8" s="49"/>
     </row>
-    <row r="9" spans="2:10" ht="15.75" thickBot="1"/>
-    <row r="10" spans="2:10" ht="16.5" thickBot="1">
+    <row r="9" spans="2:10" ht="15" thickBot="1"/>
+    <row r="10" spans="2:10" ht="16.2" thickBot="1">
       <c r="B10" s="11" t="s">
         <v>5</v>
       </c>
@@ -1203,7 +1203,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="33"/>
     </row>
-    <row r="25" spans="2:7" ht="15.75">
+    <row r="25" spans="2:7" ht="15.6">
       <c r="B25" s="36"/>
       <c r="C25" s="37"/>
       <c r="D25" s="37"/>
@@ -1239,7 +1239,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="2:7" ht="18.75">
+    <row r="29" spans="2:7" ht="18">
       <c r="B29" s="3"/>
       <c r="C29" s="38" t="s">
         <v>16</v>
@@ -1249,7 +1249,7 @@
       <c r="F29" s="40"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="2:7" ht="15.75" thickBot="1">
+    <row r="30" spans="2:7" ht="15" thickBot="1">
       <c r="B30" s="26"/>
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
@@ -1257,7 +1257,7 @@
       <c r="F30" s="27"/>
       <c r="G30" s="28"/>
     </row>
-    <row r="31" spans="2:7" ht="19.5" thickBot="1">
+    <row r="31" spans="2:7" ht="18.600000000000001" thickBot="1">
       <c r="B31" s="41" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Update Teacher Base Template.xlsx
</commit_message>
<xml_diff>
--- a/gui/template/Teacher Base Template.xlsx
+++ b/gui/template/Teacher Base Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\PycharmProjects\RueLee\bosvoiceton-gui\gui\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\Desktop\BosVoiceTon-v0.2.4-beta\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017B89D4-C528-4ACB-BE9C-6436C6830620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F01BC77-BE9E-4E61-B2D1-06FAA0AF39C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="root" sheetId="3" r:id="rId1"/>
@@ -95,7 +95,7 @@
     <t>Hours</t>
   </si>
   <si>
-    <t>4211 Wilshire Blvd., Suite 136</t>
+    <t>4055 Wilshire Blvd., Suite #400</t>
   </si>
 </sst>
 </file>
@@ -994,18 +994,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:J32"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.109375" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" customWidth="1"/>
-    <col min="4" max="4" width="24.5546875" customWidth="1"/>
+    <col min="1" max="1" width="4.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="32.4" thickBot="1">
+    <row r="1" spans="2:10" ht="33" thickBot="1">
       <c r="C1" s="7" t="s">
         <v>11</v>
       </c>
@@ -1013,13 +1013,13 @@
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="2:10" ht="18.600000000000001" thickBot="1">
+    <row r="2" spans="2:10" ht="19.5" thickBot="1">
       <c r="F2" s="14" t="s">
         <v>3</v>
       </c>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="2:10" ht="18.600000000000001" thickBot="1">
+    <row r="3" spans="2:10" ht="19.5" thickBot="1">
       <c r="B3" s="29" t="s">
         <v>19</v>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G3" s="22"/>
     </row>
-    <row r="4" spans="2:10" ht="18.600000000000001" thickBot="1">
+    <row r="4" spans="2:10" ht="19.5" thickBot="1">
       <c r="B4" s="29" t="s">
         <v>0</v>
       </c>
@@ -1050,8 +1050,8 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="2:10" ht="15" thickBot="1"/>
-    <row r="7" spans="2:10" ht="16.2" thickBot="1">
+    <row r="6" spans="2:10" ht="15.75" thickBot="1"/>
+    <row r="7" spans="2:10" ht="16.5" thickBot="1">
       <c r="B7" s="44" t="s">
         <v>4</v>
       </c>
@@ -1061,7 +1061,7 @@
       <c r="F7" s="45"/>
       <c r="G7" s="46"/>
     </row>
-    <row r="8" spans="2:10" ht="15" thickBot="1">
+    <row r="8" spans="2:10" ht="15.75" thickBot="1">
       <c r="B8" s="47"/>
       <c r="C8" s="48"/>
       <c r="D8" s="48"/>
@@ -1069,8 +1069,8 @@
       <c r="F8" s="48"/>
       <c r="G8" s="49"/>
     </row>
-    <row r="9" spans="2:10" ht="15" thickBot="1"/>
-    <row r="10" spans="2:10" ht="16.2" thickBot="1">
+    <row r="9" spans="2:10" ht="15.75" thickBot="1"/>
+    <row r="10" spans="2:10" ht="16.5" thickBot="1">
       <c r="B10" s="11" t="s">
         <v>5</v>
       </c>
@@ -1203,7 +1203,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="33"/>
     </row>
-    <row r="25" spans="2:7" ht="15.6">
+    <row r="25" spans="2:7" ht="15.75">
       <c r="B25" s="36"/>
       <c r="C25" s="37"/>
       <c r="D25" s="37"/>
@@ -1239,7 +1239,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="2:7" ht="18">
+    <row r="29" spans="2:7" ht="18.75">
       <c r="B29" s="3"/>
       <c r="C29" s="38" t="s">
         <v>16</v>
@@ -1249,7 +1249,7 @@
       <c r="F29" s="40"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="2:7" ht="15" thickBot="1">
+    <row r="30" spans="2:7" ht="15.75" thickBot="1">
       <c r="B30" s="26"/>
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
@@ -1257,7 +1257,7 @@
       <c r="F30" s="27"/>
       <c r="G30" s="28"/>
     </row>
-    <row r="31" spans="2:7" ht="18.600000000000001" thickBot="1">
+    <row r="31" spans="2:7" ht="19.5" thickBot="1">
       <c r="B31" s="41" t="s">
         <v>15</v>
       </c>

</xml_diff>